<commit_message>
📊 V9.2.1 daily run 2026-09-07_02:03
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>136.5</v>
+        <v>137.4</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>0.39</v>
+        <v>1.05</v>
       </c>
       <c r="O5" s="7" t="n">
         <v>3.55</v>
@@ -830,13 +830,13 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>33.9</v>
+        <v>33.88</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-0.62</v>
+        <v>-0.67</v>
       </c>
       <c r="O6" s="7" t="n">
         <v>0.79</v>
@@ -897,13 +897,13 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>34.88</v>
+        <v>34.8</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>-1.66</v>
+        <v>-1.89</v>
       </c>
       <c r="O7" s="7" t="n">
         <v>0.37</v>
@@ -964,13 +964,13 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>65</v>
+        <v>64.7</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-1.71</v>
+        <v>-2.16</v>
       </c>
       <c r="O8" s="7" t="n">
         <v>1.09</v>
@@ -1031,23 +1031,23 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>18</v>
+        <v>18.35</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>2.33</v>
+        <v>4.32</v>
       </c>
       <c r="O9" s="7" t="n">
-        <v>3.47</v>
+        <v>5</v>
       </c>
       <c r="P9" s="7" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
@@ -1098,19 +1098,19 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>80.16</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>0</v>
+        <v>80.3</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0.17</v>
       </c>
       <c r="O10" s="7" t="n">
-        <v>0</v>
+        <v>0.86</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>0</v>
+        <v>-2.2</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1232,23 +1232,23 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>51.6</v>
-      </c>
-      <c r="N12" s="7" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>4.65</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>0</v>
+        <v>6.98</v>
       </c>
       <c r="P12" s="7" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>36.59</v>
-      </c>
-      <c r="N13" s="7" t="n">
-        <v>0</v>
+        <v>36.44</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>-0.41</v>
       </c>
       <c r="O13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>0</v>
+        <v>-1.18</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -22184,7 +22184,7 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-09-04T02:02:51</t>
+          <t>محسوب في: 2026-09-07T02:03:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-09-21_02:04
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>37.4</v>
@@ -830,7 +830,7 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
         <v>131.6</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>122.2</v>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>58</v>
@@ -1031,7 +1031,7 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>43.84</v>
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
         <v>27.7</v>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" s="5" t="n">
         <v>21.78</v>
@@ -1232,19 +1232,19 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>78.20999999999999</v>
-      </c>
-      <c r="N12" s="7" t="n">
-        <v>0</v>
+        <v>78.05</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>-0.2</v>
       </c>
       <c r="O12" s="7" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>0</v>
+        <v>-2.31</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1299,19 +1299,19 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>25.15</v>
-      </c>
-      <c r="N13" s="7" t="n">
-        <v>0</v>
+        <v>25.1</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>-0.2</v>
       </c>
       <c r="O13" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>0</v>
+        <v>-3.58</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -24494,7 +24494,7 @@
     <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-09-18T02:03:13</t>
+          <t>محسوب في: 2026-09-21T02:04:55</t>
         </is>
       </c>
     </row>

</xml_diff>